<commit_message>
security: remove pre-filled admin credentials from login page
</commit_message>
<xml_diff>
--- a/DANH_SACH_CHIA_8_NHOM_THEO_KHOA_PHONG_BVPD.xlsx
+++ b/DANH_SACH_CHIA_8_NHOM_THEO_KHOA_PHONG_BVPD.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="397">
   <si>
     <t>BỆNH VIỆN ĐA KHOA PHƯƠNG ĐÔNG — KHÓA ĐÀO TẠO QUẢN LÝ CẤP TRUNG (80 HỌC VIÊN)</t>
   </si>
@@ -50,18 +50,21 @@
     <t>Nhóm 2</t>
   </si>
   <si>
+    <t>8 người</t>
+  </si>
+  <si>
+    <t>Khoa Cấp cứu, ICU, Khoa Ngoại, Phẫu thuật tạo hình, Gây mê hồi sức, Ngân hàng mô, Tế bào gốc, Ung bướu</t>
+  </si>
+  <si>
+    <t>Tiếp nhận cấp cứu nguy kịch &lt;= 3 phút, an toàn phẫu thuật 100%, chuyển mổ khẩn kịp thời</t>
+  </si>
+  <si>
+    <t>Nhóm 3</t>
+  </si>
+  <si>
     <t>7 người</t>
   </si>
   <si>
-    <t>Khoa Cấp cứu, ICU, Khoa Ngoại, Phẫu thuật tạo hình, Gây mê hồi sức, Ngân hàng mô, Tế bào gốc, Ung bướu</t>
-  </si>
-  <si>
-    <t>Tiếp nhận cấp cứu nguy kịch &lt;= 3 phút, an toàn phẫu thuật 100%, chuyển mổ khẩn kịp thời</t>
-  </si>
-  <si>
-    <t>Nhóm 3</t>
-  </si>
-  <si>
     <t>Khoa Nội, Khoa Nhi, Khoa Phụ sản, Y học cổ truyền, VLTL-PHCN, Hiếm muộn &amp; Nam học, CSSK toàn diện CNC</t>
   </si>
   <si>
@@ -71,10 +74,10 @@
     <t>Nhóm 4</t>
   </si>
   <si>
-    <t>5 người</t>
-  </si>
-  <si>
-    <t>Lãnh đạo Phòng Điều dưỡng toàn viện, Khoa Kiểm soát nhiễm khuẩn, Phòng Nghiệp vụ KCB &amp; BHYT, Phòng KHTH - QLCL</t>
+    <t>4 người</t>
+  </si>
+  <si>
+    <t>Lãnh đạo Phòng Điều dưỡng toàn viện, Khoa Kiểm soát nhiễm khuẩn, Phòng KHTH - QLCL</t>
   </si>
   <si>
     <t>100% điều dưỡng tuân thủ giao tiếp AIDET, kiểm soát nhiễm khuẩn &amp; quản lý chất lượng 0 lỗi</t>
@@ -353,102 +356,120 @@
     <t>NHÓM 2</t>
   </si>
   <si>
+    <t>(8 Học viên)</t>
+  </si>
+  <si>
+    <t>HV06</t>
+  </si>
+  <si>
+    <t>Ngô Thị Tuyết Mai</t>
+  </si>
+  <si>
+    <t>Khoa Cấp cứu, Hồi sức Tích cực và Chống độc</t>
+  </si>
+  <si>
+    <t>mai.ntt06@phuongdonghospital.vn</t>
+  </si>
+  <si>
+    <t>HV10</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Hồng Ngân</t>
+  </si>
+  <si>
+    <t>Kỹ thuật viên phụ trách</t>
+  </si>
+  <si>
+    <t>Ngân hàng Mô Phương Đông</t>
+  </si>
+  <si>
+    <t>ngan.nth10@phuongdonghospital.vn</t>
+  </si>
+  <si>
+    <t>HV11</t>
+  </si>
+  <si>
+    <t>Trần Hồng Ngân</t>
+  </si>
+  <si>
+    <t>Trung tâm Y học Tái tạo và Trị liệu Tế bào</t>
+  </si>
+  <si>
+    <t>ngan.th11@phuongdonghospital.vn</t>
+  </si>
+  <si>
+    <t>HV12</t>
+  </si>
+  <si>
+    <t>Nguyễn Đình Dương</t>
+  </si>
+  <si>
+    <t>Trung tâm Ung bướu, Xạ trị và Y học hạt nhân Quốc tế Phương Đông</t>
+  </si>
+  <si>
+    <t>duong.nd12@phuongdonghospital.vn</t>
+  </si>
+  <si>
+    <t>HV13</t>
+  </si>
+  <si>
+    <t>Vũ Thị Hải Ngọc</t>
+  </si>
+  <si>
+    <t>Điều dưỡng phó</t>
+  </si>
+  <si>
+    <t>Khoa Ngoại</t>
+  </si>
+  <si>
+    <t>ngoc.vth13@phuongdonghospital.vn</t>
+  </si>
+  <si>
+    <t>HV14</t>
+  </si>
+  <si>
+    <t>Nông Thị Khánh Linh</t>
+  </si>
+  <si>
+    <t>Khoa Phẫu thuật tạo hình Thẩm mỹ</t>
+  </si>
+  <si>
+    <t>linh.ntk14@phuongdonghospital.vn</t>
+  </si>
+  <si>
+    <t>HV15</t>
+  </si>
+  <si>
+    <t>Vũ Thị Thanh Mai</t>
+  </si>
+  <si>
+    <t>Khoa Gây mê hồi sức</t>
+  </si>
+  <si>
+    <t>mai.vtt15@phuongdonghospital.vn</t>
+  </si>
+  <si>
+    <t>HV26</t>
+  </si>
+  <si>
+    <t>Bùi Mỹ Lương</t>
+  </si>
+  <si>
+    <t>Trưởng phòng</t>
+  </si>
+  <si>
+    <t>Phòng Nghiệp vụ Khám chữa bệnh và Bảo hiểm Y tế</t>
+  </si>
+  <si>
+    <t>luong.bm26@phuongdonghospital.vn</t>
+  </si>
+  <si>
+    <t>NHÓM 3</t>
+  </si>
+  <si>
     <t>(7 Học viên)</t>
   </si>
   <si>
-    <t>HV06</t>
-  </si>
-  <si>
-    <t>Ngô Thị Tuyết Mai</t>
-  </si>
-  <si>
-    <t>Khoa Cấp cứu, Hồi sức Tích cực và Chống độc</t>
-  </si>
-  <si>
-    <t>mai.ntt06@phuongdonghospital.vn</t>
-  </si>
-  <si>
-    <t>HV10</t>
-  </si>
-  <si>
-    <t>Nguyễn Thị Hồng Ngân</t>
-  </si>
-  <si>
-    <t>Kỹ thuật viên phụ trách</t>
-  </si>
-  <si>
-    <t>Ngân hàng Mô Phương Đông</t>
-  </si>
-  <si>
-    <t>ngan.nth10@phuongdonghospital.vn</t>
-  </si>
-  <si>
-    <t>HV11</t>
-  </si>
-  <si>
-    <t>Trần Hồng Ngân</t>
-  </si>
-  <si>
-    <t>Trung tâm Y học Tái tạo và Trị liệu Tế bào</t>
-  </si>
-  <si>
-    <t>ngan.th11@phuongdonghospital.vn</t>
-  </si>
-  <si>
-    <t>HV12</t>
-  </si>
-  <si>
-    <t>Nguyễn Đình Dương</t>
-  </si>
-  <si>
-    <t>Trung tâm Ung bướu, Xạ trị và Y học hạt nhân Quốc tế Phương Đông</t>
-  </si>
-  <si>
-    <t>duong.nd12@phuongdonghospital.vn</t>
-  </si>
-  <si>
-    <t>HV13</t>
-  </si>
-  <si>
-    <t>Vũ Thị Hải Ngọc</t>
-  </si>
-  <si>
-    <t>Điều dưỡng phó</t>
-  </si>
-  <si>
-    <t>Khoa Ngoại</t>
-  </si>
-  <si>
-    <t>ngoc.vth13@phuongdonghospital.vn</t>
-  </si>
-  <si>
-    <t>HV14</t>
-  </si>
-  <si>
-    <t>Nông Thị Khánh Linh</t>
-  </si>
-  <si>
-    <t>Khoa Phẫu thuật tạo hình Thẩm mỹ</t>
-  </si>
-  <si>
-    <t>linh.ntk14@phuongdonghospital.vn</t>
-  </si>
-  <si>
-    <t>HV15</t>
-  </si>
-  <si>
-    <t>Vũ Thị Thanh Mai</t>
-  </si>
-  <si>
-    <t>Khoa Gây mê hồi sức</t>
-  </si>
-  <si>
-    <t>mai.vtt15@phuongdonghospital.vn</t>
-  </si>
-  <si>
-    <t>NHÓM 3</t>
-  </si>
-  <si>
     <t>HV07</t>
   </si>
   <si>
@@ -539,7 +560,7 @@
     <t>NHÓM 4</t>
   </si>
   <si>
-    <t>(5 Học viên)</t>
+    <t>(4 Học viên)</t>
   </si>
   <si>
     <t>HV25</t>
@@ -552,21 +573,6 @@
   </si>
   <si>
     <t>thuy.np25@phuongdonghospital.vn</t>
-  </si>
-  <si>
-    <t>HV26</t>
-  </si>
-  <si>
-    <t>Bùi Mỹ Lương</t>
-  </si>
-  <si>
-    <t>Trưởng phòng</t>
-  </si>
-  <si>
-    <t>Phòng Nghiệp vụ Khám chữa bệnh và Bảo hiểm Y tế</t>
-  </si>
-  <si>
-    <t>luong.bm26@phuongdonghospital.vn</t>
   </si>
   <si>
     <t>HV28</t>
@@ -1882,83 +1888,83 @@
         <v>15</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1988,7 +1994,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2000,7 +2006,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2012,36 +2018,36 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="11"/>
@@ -2058,22 +2064,22 @@
         <v>7</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2084,22 +2090,22 @@
         <v>7</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2110,22 +2116,22 @@
         <v>7</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2136,22 +2142,22 @@
         <v>7</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H9" s="19" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2162,22 +2168,22 @@
         <v>7</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2188,22 +2194,22 @@
         <v>7</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H11" s="19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2214,22 +2220,22 @@
         <v>7</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2240,22 +2246,22 @@
         <v>7</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H13" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2266,22 +2272,22 @@
         <v>7</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2292,22 +2298,22 @@
         <v>7</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H15" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2318,22 +2324,22 @@
         <v>7</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2344,22 +2350,22 @@
         <v>7</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H17" s="19" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2370,22 +2376,22 @@
         <v>7</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2396,22 +2402,22 @@
         <v>7</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H19" s="19" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2422,30 +2428,30 @@
         <v>7</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
@@ -2462,22 +2468,22 @@
         <v>11</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H22" s="15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2488,22 +2494,22 @@
         <v>11</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H23" s="19" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2514,22 +2520,22 @@
         <v>11</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2540,22 +2546,22 @@
         <v>11</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H25" s="19" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2566,22 +2572,22 @@
         <v>11</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H26" s="15" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2592,22 +2598,22 @@
         <v>11</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H27" s="19" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2618,370 +2624,370 @@
         <v>11</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H28" s="15" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="29" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="B29" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
-    </row>
-    <row r="30" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="12">
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="16">
+        <v>8</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="E29" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="F29" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="G29" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="H29" s="19" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="B30" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="23"/>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="12">
         <v>1</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B31" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C30" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="D30" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="E30" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="F30" s="15" t="s">
+      <c r="C31" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="F31" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="G31" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H31" s="15" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="16">
+        <v>2</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C32" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="D32" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="E32" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="F32" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="G32" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="H32" s="19" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="12">
+        <v>3</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="G33" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H33" s="15" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="16">
+        <v>4</v>
+      </c>
+      <c r="B34" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C34" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="D34" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="E34" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="F34" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="G34" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="H34" s="19" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="12">
+        <v>5</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="F35" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="G35" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="16">
+        <v>6</v>
+      </c>
+      <c r="B36" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="D36" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="E36" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="F36" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="G36" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="H36" s="19" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="12">
+        <v>7</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="E37" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="F37" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="G37" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H37" s="15" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="24" t="s">
+        <v>181</v>
+      </c>
+      <c r="B38" s="25" t="s">
+        <v>182</v>
+      </c>
+      <c r="C38" s="25"/>
+      <c r="D38" s="25"/>
+      <c r="E38" s="25"/>
+      <c r="F38" s="25"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="25"/>
+    </row>
+    <row r="39" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="12">
+        <v>1</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="E39" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="F39" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="G39" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H39" s="15" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="40" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="16">
+        <v>2</v>
+      </c>
+      <c r="B40" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C40" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="D40" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="E40" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="G30" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="H30" s="15" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="31" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="16">
-        <v>2</v>
-      </c>
-      <c r="B31" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="C31" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="D31" s="18" t="s">
-        <v>150</v>
-      </c>
-      <c r="E31" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="F31" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="G31" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="H31" s="19" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="32" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="12">
+      <c r="F40" s="19" t="s">
+        <v>189</v>
+      </c>
+      <c r="G40" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="H40" s="19" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="41" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="12">
         <v>3</v>
       </c>
-      <c r="B32" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="D32" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="E32" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="F32" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="G32" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="H32" s="15" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="33" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="16">
+      <c r="B41" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="F41" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="G41" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H41" s="15" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="42" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="16">
         <v>4</v>
       </c>
-      <c r="B33" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="C33" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="D33" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="E33" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="F33" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="G33" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="H33" s="19" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="12">
-        <v>5</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>161</v>
-      </c>
-      <c r="D34" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="E34" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="F34" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="G34" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="H34" s="15" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="35" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="16">
-        <v>6</v>
-      </c>
-      <c r="B35" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="C35" s="17" t="s">
-        <v>166</v>
-      </c>
-      <c r="D35" s="18" t="s">
-        <v>167</v>
-      </c>
-      <c r="E35" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="F35" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="G35" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="H35" s="19" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="36" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="12">
-        <v>7</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>170</v>
-      </c>
-      <c r="D36" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="E36" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="F36" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="G36" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="H36" s="15" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="37" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="24" t="s">
-        <v>174</v>
-      </c>
-      <c r="B37" s="25" t="s">
-        <v>175</v>
-      </c>
-      <c r="C37" s="25"/>
-      <c r="D37" s="25"/>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25"/>
-      <c r="G37" s="25"/>
-      <c r="H37" s="25"/>
-    </row>
-    <row r="38" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="12">
-        <v>1</v>
-      </c>
-      <c r="B38" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C38" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D38" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="E38" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="F38" s="15" t="s">
-        <v>178</v>
-      </c>
-      <c r="G38" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="H38" s="15" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="39" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="16">
-        <v>2</v>
-      </c>
-      <c r="B39" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C39" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="D39" s="18" t="s">
-        <v>181</v>
-      </c>
-      <c r="E39" s="19" t="s">
-        <v>182</v>
-      </c>
-      <c r="F39" s="19" t="s">
-        <v>183</v>
-      </c>
-      <c r="G39" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="H39" s="19" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="40" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="12">
-        <v>3</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="D40" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="E40" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="F40" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="G40" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="H40" s="15" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="41" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="16">
-        <v>4</v>
-      </c>
-      <c r="B41" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C41" s="17" t="s">
-        <v>189</v>
-      </c>
-      <c r="D41" s="18" t="s">
-        <v>190</v>
-      </c>
-      <c r="E41" s="19" t="s">
-        <v>191</v>
-      </c>
-      <c r="F41" s="19" t="s">
-        <v>192</v>
-      </c>
-      <c r="G41" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="H41" s="19" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="42" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="12">
-        <v>5</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C42" s="13" t="s">
+      <c r="B42" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="D42" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="E42" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="F42" s="19" t="s">
         <v>194</v>
       </c>
-      <c r="D42" s="14" t="s">
-        <v>195</v>
-      </c>
-      <c r="E42" s="15" t="s">
-        <v>196</v>
-      </c>
-      <c r="F42" s="15" t="s">
-        <v>192</v>
-      </c>
-      <c r="G42" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="H42" s="15" t="s">
-        <v>197</v>
+      <c r="G42" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="H42" s="19" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="43" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="26" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B43" s="27" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C43" s="27"/>
       <c r="D43" s="27"/>
@@ -2995,25 +3001,25 @@
         <v>1</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="F44" s="15" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G44" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H44" s="15" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="45" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3021,25 +3027,25 @@
         <v>2</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C45" s="17" t="s">
+        <v>206</v>
+      </c>
+      <c r="D45" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="E45" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="F45" s="19" t="s">
         <v>204</v>
       </c>
-      <c r="D45" s="18" t="s">
-        <v>205</v>
-      </c>
-      <c r="E45" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="F45" s="19" t="s">
-        <v>202</v>
-      </c>
       <c r="G45" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H45" s="19" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="46" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3047,25 +3053,25 @@
         <v>3</v>
       </c>
       <c r="B46" s="12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="F46" s="15" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G46" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H46" s="15" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="47" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3073,25 +3079,25 @@
         <v>4</v>
       </c>
       <c r="B47" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C47" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="D47" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="E47" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="F47" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="D47" s="18" t="s">
-        <v>213</v>
-      </c>
-      <c r="E47" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="F47" s="19" t="s">
-        <v>210</v>
-      </c>
       <c r="G47" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="48" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3099,25 +3105,25 @@
         <v>5</v>
       </c>
       <c r="B48" s="12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E48" s="15" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="F48" s="15" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G48" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H48" s="15" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="49" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3125,25 +3131,25 @@
         <v>6</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C49" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="D49" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="E49" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="F49" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="D49" s="18" t="s">
-        <v>220</v>
-      </c>
-      <c r="E49" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="F49" s="19" t="s">
-        <v>217</v>
-      </c>
       <c r="G49" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H49" s="19" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="50" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3151,25 +3157,25 @@
         <v>7</v>
       </c>
       <c r="B50" s="12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E50" s="15" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="F50" s="15" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G50" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H50" s="15" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="51" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3177,25 +3183,25 @@
         <v>8</v>
       </c>
       <c r="B51" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C51" s="17" t="s">
+        <v>228</v>
+      </c>
+      <c r="D51" s="18" t="s">
+        <v>229</v>
+      </c>
+      <c r="E51" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="F51" s="19" t="s">
         <v>226</v>
       </c>
-      <c r="D51" s="18" t="s">
-        <v>227</v>
-      </c>
-      <c r="E51" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="F51" s="19" t="s">
-        <v>224</v>
-      </c>
       <c r="G51" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H51" s="19" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="52" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3203,25 +3209,25 @@
         <v>9</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F52" s="15" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="G52" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H52" s="15" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="53" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3229,25 +3235,25 @@
         <v>10</v>
       </c>
       <c r="B53" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C53" s="17" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D53" s="18" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E53" s="19" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F53" s="19" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H53" s="19" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="54" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3255,25 +3261,25 @@
         <v>11</v>
       </c>
       <c r="B54" s="12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D54" s="14" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="F54" s="15" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G54" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H54" s="15" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="55" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3281,25 +3287,25 @@
         <v>12</v>
       </c>
       <c r="B55" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C55" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="D55" s="18" t="s">
+        <v>246</v>
+      </c>
+      <c r="E55" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="F55" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="D55" s="18" t="s">
-        <v>244</v>
-      </c>
-      <c r="E55" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="F55" s="19" t="s">
-        <v>241</v>
-      </c>
       <c r="G55" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H55" s="19" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="56" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3307,33 +3313,33 @@
         <v>13</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D56" s="14" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F56" s="15" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="G56" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H56" s="15" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="57" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="28" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B57" s="29" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C57" s="29"/>
       <c r="D57" s="29"/>
@@ -3347,25 +3353,25 @@
         <v>1</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D58" s="14" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E58" s="15" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F58" s="15" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="G58" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H58" s="15" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="59" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3373,25 +3379,25 @@
         <v>2</v>
       </c>
       <c r="B59" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C59" s="17" t="s">
+        <v>258</v>
+      </c>
+      <c r="D59" s="18" t="s">
+        <v>259</v>
+      </c>
+      <c r="E59" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="F59" s="19" t="s">
         <v>256</v>
       </c>
-      <c r="D59" s="18" t="s">
-        <v>257</v>
-      </c>
-      <c r="E59" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="F59" s="19" t="s">
-        <v>254</v>
-      </c>
       <c r="G59" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H59" s="19" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="60" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3399,25 +3405,25 @@
         <v>3</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D60" s="14" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E60" s="15" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F60" s="15" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="G60" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H60" s="15" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="61" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3425,25 +3431,25 @@
         <v>4</v>
       </c>
       <c r="B61" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C61" s="17" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D61" s="18" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E61" s="19" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F61" s="19" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="G61" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H61" s="19" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="62" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3451,25 +3457,25 @@
         <v>5</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D62" s="14" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E62" s="15" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="F62" s="15" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="G62" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H62" s="15" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="63" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3477,25 +3483,25 @@
         <v>6</v>
       </c>
       <c r="B63" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C63" s="17" t="s">
+        <v>274</v>
+      </c>
+      <c r="D63" s="18" t="s">
+        <v>275</v>
+      </c>
+      <c r="E63" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="F63" s="19" t="s">
         <v>272</v>
       </c>
-      <c r="D63" s="18" t="s">
-        <v>273</v>
-      </c>
-      <c r="E63" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="F63" s="19" t="s">
-        <v>270</v>
-      </c>
       <c r="G63" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H63" s="19" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="64" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3503,25 +3509,25 @@
         <v>7</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D64" s="14" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="E64" s="15" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="F64" s="15" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="G64" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H64" s="15" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="65" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3529,25 +3535,25 @@
         <v>8</v>
       </c>
       <c r="B65" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C65" s="17" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D65" s="18" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E65" s="19" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="F65" s="19" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="G65" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H65" s="19" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="66" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3555,25 +3561,25 @@
         <v>9</v>
       </c>
       <c r="B66" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C66" s="13" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D66" s="14" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E66" s="15" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="F66" s="15" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="G66" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H66" s="15" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="67" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3581,25 +3587,25 @@
         <v>10</v>
       </c>
       <c r="B67" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C67" s="17" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D67" s="18" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E67" s="19" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F67" s="19" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="G67" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H67" s="19" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="68" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3607,25 +3613,25 @@
         <v>11</v>
       </c>
       <c r="B68" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="D68" s="14" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E68" s="15" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="F68" s="15" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="G68" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H68" s="15" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="69" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3633,25 +3639,25 @@
         <v>12</v>
       </c>
       <c r="B69" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C69" s="17" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D69" s="18" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E69" s="19" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F69" s="19" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="G69" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H69" s="19" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="70" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3659,33 +3665,33 @@
         <v>13</v>
       </c>
       <c r="B70" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D70" s="14" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E70" s="15" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F70" s="15" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="G70" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H70" s="15" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="71" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="30" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B71" s="31" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="C71" s="31"/>
       <c r="D71" s="31"/>
@@ -3699,25 +3705,25 @@
         <v>1</v>
       </c>
       <c r="B72" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C72" s="13" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D72" s="14" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E72" s="15" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="F72" s="15" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="G72" s="12" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H72" s="15" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="73" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3725,25 +3731,25 @@
         <v>2</v>
       </c>
       <c r="B73" s="16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C73" s="17" t="s">
+        <v>312</v>
+      </c>
+      <c r="D73" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="E73" s="19" t="s">
+        <v>314</v>
+      </c>
+      <c r="F73" s="19" t="s">
+        <v>315</v>
+      </c>
+      <c r="G73" s="16" t="s">
         <v>310</v>
       </c>
-      <c r="D73" s="18" t="s">
-        <v>311</v>
-      </c>
-      <c r="E73" s="19" t="s">
-        <v>312</v>
-      </c>
-      <c r="F73" s="19" t="s">
-        <v>313</v>
-      </c>
-      <c r="G73" s="16" t="s">
-        <v>308</v>
-      </c>
       <c r="H73" s="19" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="74" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3751,25 +3757,25 @@
         <v>3</v>
       </c>
       <c r="B74" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C74" s="13" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D74" s="14" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E74" s="15" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F74" s="15" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="G74" s="12" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H74" s="15" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="75" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3777,25 +3783,25 @@
         <v>4</v>
       </c>
       <c r="B75" s="16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C75" s="17" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D75" s="18" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E75" s="19" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="F75" s="19" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H75" s="19" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="76" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3803,25 +3809,25 @@
         <v>5</v>
       </c>
       <c r="B76" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D76" s="14" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="E76" s="15" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="F76" s="15" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="G76" s="12" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H76" s="15" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="77" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3829,25 +3835,25 @@
         <v>6</v>
       </c>
       <c r="B77" s="16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C77" s="17" t="s">
+        <v>331</v>
+      </c>
+      <c r="D77" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="E77" s="19" t="s">
+        <v>328</v>
+      </c>
+      <c r="F77" s="19" t="s">
         <v>329</v>
       </c>
-      <c r="D77" s="18" t="s">
-        <v>330</v>
-      </c>
-      <c r="E77" s="19" t="s">
-        <v>326</v>
-      </c>
-      <c r="F77" s="19" t="s">
-        <v>327</v>
-      </c>
       <c r="G77" s="16" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H77" s="19" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="78" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3855,33 +3861,33 @@
         <v>7</v>
       </c>
       <c r="B78" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D78" s="14" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E78" s="15" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="F78" s="15" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="G78" s="12" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H78" s="15" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="79" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="32" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B79" s="33" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C79" s="33"/>
       <c r="D79" s="33"/>
@@ -3895,25 +3901,25 @@
         <v>1</v>
       </c>
       <c r="B80" s="12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D80" s="14" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="E80" s="15" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="F80" s="15" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="G80" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H80" s="15" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="81" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3921,25 +3927,25 @@
         <v>2</v>
       </c>
       <c r="B81" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C81" s="17" t="s">
+        <v>346</v>
+      </c>
+      <c r="D81" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="E81" s="19" t="s">
+        <v>348</v>
+      </c>
+      <c r="F81" s="19" t="s">
+        <v>343</v>
+      </c>
+      <c r="G81" s="16" t="s">
         <v>344</v>
       </c>
-      <c r="D81" s="18" t="s">
-        <v>345</v>
-      </c>
-      <c r="E81" s="19" t="s">
-        <v>346</v>
-      </c>
-      <c r="F81" s="19" t="s">
-        <v>341</v>
-      </c>
-      <c r="G81" s="16" t="s">
-        <v>342</v>
-      </c>
       <c r="H81" s="19" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="82" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3947,25 +3953,25 @@
         <v>3</v>
       </c>
       <c r="B82" s="12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C82" s="13" t="s">
+        <v>350</v>
+      </c>
+      <c r="D82" s="14" t="s">
+        <v>351</v>
+      </c>
+      <c r="E82" s="15" t="s">
         <v>348</v>
       </c>
-      <c r="D82" s="14" t="s">
-        <v>349</v>
-      </c>
-      <c r="E82" s="15" t="s">
-        <v>346</v>
-      </c>
       <c r="F82" s="15" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="G82" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H82" s="15" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="83" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3973,25 +3979,25 @@
         <v>4</v>
       </c>
       <c r="B83" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C83" s="17" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D83" s="18" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E83" s="19" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="F83" s="19" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="G83" s="16" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H83" s="19" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="84" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3999,25 +4005,25 @@
         <v>5</v>
       </c>
       <c r="B84" s="12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C84" s="13" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D84" s="14" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="E84" s="15" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="F84" s="15" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="G84" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H84" s="15" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="85" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4025,25 +4031,25 @@
         <v>6</v>
       </c>
       <c r="B85" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C85" s="17" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D85" s="18" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E85" s="19" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F85" s="19" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="G85" s="16" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H85" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="86" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4051,25 +4057,25 @@
         <v>7</v>
       </c>
       <c r="B86" s="12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C86" s="13" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D86" s="14" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E86" s="15" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="F86" s="15" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="G86" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H86" s="15" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="87" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4077,25 +4083,25 @@
         <v>8</v>
       </c>
       <c r="B87" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C87" s="17" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D87" s="18" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E87" s="19" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F87" s="19" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="G87" s="16" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H87" s="19" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="88" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4103,25 +4109,25 @@
         <v>9</v>
       </c>
       <c r="B88" s="12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C88" s="13" t="s">
+        <v>375</v>
+      </c>
+      <c r="D88" s="14" t="s">
+        <v>376</v>
+      </c>
+      <c r="E88" s="15" t="s">
+        <v>377</v>
+      </c>
+      <c r="F88" s="15" t="s">
         <v>373</v>
       </c>
-      <c r="D88" s="14" t="s">
-        <v>374</v>
-      </c>
-      <c r="E88" s="15" t="s">
-        <v>375</v>
-      </c>
-      <c r="F88" s="15" t="s">
-        <v>371</v>
-      </c>
       <c r="G88" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H88" s="15" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="89" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4129,25 +4135,25 @@
         <v>10</v>
       </c>
       <c r="B89" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C89" s="17" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D89" s="18" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="E89" s="19" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F89" s="19" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="G89" s="16" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H89" s="19" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="90" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4155,25 +4161,25 @@
         <v>11</v>
       </c>
       <c r="B90" s="12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C90" s="13" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D90" s="14" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="E90" s="15" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="F90" s="15" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="G90" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H90" s="15" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="91" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4181,25 +4187,25 @@
         <v>12</v>
       </c>
       <c r="B91" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C91" s="17" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="D91" s="18" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="E91" s="19" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="F91" s="19" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G91" s="16" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H91" s="19" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="92" ht="24" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4207,25 +4213,25 @@
         <v>13</v>
       </c>
       <c r="B92" s="12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C92" s="13" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D92" s="14" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E92" s="15" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F92" s="15" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="G92" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H92" s="15" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -4234,8 +4240,8 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="B21:H21"/>
-    <mergeCell ref="B29:H29"/>
-    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="B30:H30"/>
+    <mergeCell ref="B38:H38"/>
     <mergeCell ref="B43:H43"/>
     <mergeCell ref="B57:H57"/>
     <mergeCell ref="B71:H71"/>

</xml_diff>